<commit_message>
Add cleaned final dataset for Tan Son Nhat Airport communications
- Introduced a new CSV file containing cleaned and normalized communication transcripts from Tan Son Nhat Airport.
- The dataset includes timestamps, callsigns, and various cleaned text versions for improved readability and analysis.
- Ensured consistency in formatting and terminology across all entries.
</commit_message>
<xml_diff>
--- a/VJC1225 and 2 more.xlsx
+++ b/VJC1225 and 2 more.xlsx
@@ -596,8 +596,10 @@
       <c r="B6" s="2">
         <v>6.9444444444444447E-4</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PILOT</t>
+        </is>
       </c>
       <c r="D6" t="s">
         <v>8</v>

</xml_diff>